<commit_message>
add net lab - messaging
</commit_message>
<xml_diff>
--- a/earth-pipeline/HowUnitTestPipelineWorks.xlsx
+++ b/earth-pipeline/HowUnitTestPipelineWorks.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\cuifawei-d\documents\earth-pipeline\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{494B7578-0692-457D-BAA1-D775985C466F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA0070C0-D259-4D5D-9ECB-AEFE439A4C98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="51840" windowHeight="21120" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,8 @@
     <sheet name="pipeline" sheetId="9" r:id="rId7"/>
     <sheet name="pipeline-PR_Pipeline.yml" sheetId="10" r:id="rId8"/>
     <sheet name="PR_Gate.yml" sheetId="11" r:id="rId9"/>
-    <sheet name="pipeline-Nunit" sheetId="3" r:id="rId10"/>
+    <sheet name="Resharper" sheetId="12" r:id="rId10"/>
+    <sheet name="pipeline-Nunit" sheetId="3" r:id="rId11"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -34,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="319" uniqueCount="222">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="335" uniqueCount="223">
   <si>
     <r>
       <t xml:space="preserve">VS 在加载项目时，尝试导入一个共享的 MSBuild 目标文件 </t>
@@ -2620,6 +2621,9 @@
   <si>
     <t>变量组，有很多变量在这里</t>
     <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>PR_Gate.yml</t>
   </si>
 </sst>
 </file>
@@ -2960,6 +2964,143 @@
         <a:xfrm>
           <a:off x="0" y="15087600"/>
           <a:ext cx="8914286" cy="4533333"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing10.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>131445</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>456381</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>10910</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{67E6B0C0-3481-07FA-8616-17ED29A6E296}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="1160145"/>
+          <a:ext cx="6552381" cy="4165715"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>38</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>465371</xdr:colOff>
+      <xdr:row>80</xdr:row>
+      <xdr:rowOff>27671</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E8527176-087F-1B13-ABE4-BF31EE88E469}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="609600" y="6515100"/>
+          <a:ext cx="10828571" cy="7228571"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>83</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>503390</xdr:colOff>
+      <xdr:row>123</xdr:row>
+      <xdr:rowOff>37238</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D51641D6-067C-B26D-901E-E4448E04C178}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="14230350"/>
+          <a:ext cx="11476190" cy="6895238"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -4242,23 +4383,23 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>0</xdr:col>
+      <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>131445</xdr:rowOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>456381</xdr:colOff>
-      <xdr:row>31</xdr:row>
-      <xdr:rowOff>10910</xdr:rowOff>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>103848</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>161626</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="2" name="Picture 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{67E6B0C0-3481-07FA-8616-17ED29A6E296}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{62163240-C3FE-0431-E9E3-51BF88DD69C8}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -4274,96 +4415,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="0" y="1160145"/>
-          <a:ext cx="6552381" cy="4165715"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>38</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>18</xdr:col>
-      <xdr:colOff>465371</xdr:colOff>
-      <xdr:row>80</xdr:row>
-      <xdr:rowOff>27671</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Picture 2">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E8527176-087F-1B13-ABE4-BF31EE88E469}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="609600" y="6515100"/>
-          <a:ext cx="10828571" cy="7228571"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>83</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>18</xdr:col>
-      <xdr:colOff>503390</xdr:colOff>
-      <xdr:row>123</xdr:row>
-      <xdr:rowOff>37238</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="Picture 3">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D51641D6-067C-B26D-901E-E4448E04C178}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="14230350"/>
-          <a:ext cx="11476190" cy="6895238"/>
+          <a:off x="609600" y="3429000"/>
+          <a:ext cx="7419048" cy="2390476"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -5368,6 +5421,98 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A26ABD03-4BD3-4CD9-842A-3E9B9DC60DD0}">
+  <dimension ref="A2:B17"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="2" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B3" s="13" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B4" s="13" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B5" s="13" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B6" s="13" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B7" s="13" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B8" s="13" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B9" s="13" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B10" s="13" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B11" s="13" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B12" s="13" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B13" s="13" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B14" s="13" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B15" s="13" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B16" s="13" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="17" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B17" s="13" t="s">
+        <v>218</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{32137F47-3F32-4937-AF61-315CDE07C17B}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>

</xml_diff>